<commit_message>
Swap restaurant for horse retirement stable; farm-stay to annual rental
Removes the restaurant revenue/cost lines and capex, adds a 20-stall
horse retirement/boarding stable (same boarding-fee model as the horse
sanctuary plan). Farm-stay units now rent annually to families instead
of nightly to tourists, to genuinely test commitment during the lease
period rather than run hotel-style occupancy.

Flags the resulting finding: 5-year operating profit no longer comes
close to self-funding the Year 5 land purchase (cumulative cash position
after buying the land drops from ~-41.0M to ~-123.1M), so the plan now
depends on external financing at Year 5 rather than being self-funded.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T2AH8DfmywYakYgEQMQoZc
</commit_message>
<xml_diff>
--- a/business-plan/rent-to-buy-model/Farm_De_Rai_Rent_To_Buy_Model.xlsx
+++ b/business-plan/rent-to-buy-model/Farm_De_Rai_Rent_To_Buy_Model.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="135">
   <si>
     <t xml:space="preserve">Farm De Rai — Rent-to-Buy Model</t>
   </si>
@@ -33,10 +33,16 @@
     <t xml:space="preserve">How to use this workbook</t>
   </si>
   <si>
-    <t xml:space="preserve">This is a standalone ALTERNATIVE to the horse sanctuary / land-purchase plan — a different business</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(farm-stay + EV charging + restaurant) on the same 42 rai, leased first and purchased at Year 5.</t>
+    <t xml:space="preserve">This is the lease-first path to buying the 42 rai next to Farm De Lek: a farm-stay + EV charging +</t>
+  </si>
+  <si>
+    <t xml:space="preserve">horse retirement stable business, run on leased land, then purchased outright at Year 5. Five years of</t>
+  </si>
+  <si>
+    <t xml:space="preserve">operating history is the test — proof of the business and the commitment needed to close the purchase.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Once bought, 12 of the 42 rai are gifted to the horse sanctuary; the remaining 30 stay with this business.</t>
   </si>
   <si>
     <t xml:space="preserve">Change any blue number and every sheet, including the Summary chart, recalculates.</t>
@@ -60,10 +66,10 @@
     <t xml:space="preserve">Sheet guide</t>
   </si>
   <si>
-    <t xml:space="preserve">   Assumptions — land rent, occupancy/utilization ramps, pricing, staffing, and the Year-5 buy/sell terms</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   Capex        — the ~฿ 38.0M upfront build cost, itemized (no land purchase — that happens at Year 5)</t>
+    <t xml:space="preserve">   Assumptions — land rent, farm-stay/EV/charging/horse-boarding ramps, pricing, staffing, and the Year-5 buy/sell terms</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Capex        — the ~฿ 46.0M upfront build cost, itemized (no land purchase — that happens at Year 5)</t>
   </si>
   <si>
     <t xml:space="preserve">   Operating P&amp;L — 5-year revenue (4 streams) and operating cost</t>
@@ -102,45 +108,57 @@
     <t xml:space="preserve">Lease start date</t>
   </si>
   <si>
-    <t xml:space="preserve">FARM-STAY (20 pre-built units)</t>
+    <t xml:space="preserve">FARM-STAY HOMES (20 pre-built units, rented ANNUALLY to test commitment)</t>
   </si>
   <si>
     <t xml:space="preserve">Units (count)</t>
   </si>
   <si>
+    <t xml:space="preserve">Annual rent per unit (THB/year)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rented by the year, not the night — the point is to sign up committed families early, not run a hotel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Assumption</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Year 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Year 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Year 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Year 4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Year 5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Notes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Units occupied (count, out of 20)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ramps up as families commit — full occupancy by Year 5, when the land purchase closes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EV PARK &amp; STAY (10 bays)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bays (count)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Nightly rate (THB)</t>
   </si>
   <si>
-    <t xml:space="preserve">Assumption</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Year 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Year 2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Year 3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Year 4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Year 5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Notes</t>
-  </si>
-  <si>
     <t xml:space="preserve">Occupancy %</t>
   </si>
   <si>
-    <t xml:space="preserve">EV PARK &amp; STAY (10 bays)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bays (count)</t>
-  </si>
-  <si>
     <t xml:space="preserve">FAST CHARGING (5 chargers)</t>
   </si>
   <si>
@@ -159,148 +177,163 @@
     <t xml:space="preserve">Sessions per charger per day</t>
   </si>
   <si>
-    <t xml:space="preserve">RESTAURANT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Average spend per cover (THB)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Food &amp; beverage cost (% of restaurant revenue)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Covers per day</t>
+    <t xml:space="preserve">HORSE RETIREMENT STABLE (up to 20 horses, paid boarding)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Boarding fee (THB / horse / month)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Feed / routine care cost (THB / horse / month)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vet fees are billed directly to the horse owner — not in this model</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Horses in care (capped at 20)</t>
   </si>
   <si>
     <t xml:space="preserve">OPERATING COSTS (per year)</t>
   </si>
   <si>
+    <t xml:space="preserve">Staff (farm-stay, EV/charger, reception — no restaurant team)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stable caretakers (grooms, farrier support)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Utilities</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Marketing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Admin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Maintenance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAPEX (one-time)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20 pre-built farm-stay units (THB/unit)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Site infrastructure (roads, water, electrical backbone)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EV park-and-stay pad (THB/pad)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DC fast charger, incl. install (THB/charger)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Horse stable barn (20 stalls) + tack/feed room</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Paddock &amp; perimeter fencing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Initial stable fit-out &amp; onboarding</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reception/admin building</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Equipment &amp; vehicles</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Working capital reserve</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contingency + legal/permits/lease deposit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">YEAR 5 — TERMINAL TRANSACTION (sell houses, buy land)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Farm-stay unit resale value (% of original cost)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Land purchase price at Year 5 (THB, total 42 rai)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Placeholder: ~2.3M/rai per the owner's earlier pricing — confirm the actual negotiated price</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rent credited toward purchase price (% of 5-yr rent paid)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A rent-to-own term worth negotiating with the owner</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rai gifted to the sanctuary after purchase</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Informational only — no cost impact here; the remaining rai stay with the tourism business</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Capital Expenditure</t>
+  </si>
+  <si>
+    <t xml:space="preserve">~฿ 46.0M upfront — no land purchase in this phase</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Item</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amount (THB)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">% of total</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20 pre-built farm-stay units</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10 EV park-and-stay pads</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5 DC fast chargers (incl. install)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOTAL CAPEX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5-Year Operating Plan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Farm-stay homes (annual rental) + EV park &amp; charging + horse retirement stable, on leased land</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REVENUE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Farm-stay homes (units occupied × annual rent)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EV park &amp; stay (bays × occ × rate × 365)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fast charging (chargers × sessions/day × kWh × price × 365)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Horse retirement boarding (horses × boarding fee × 12)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOTAL REVENUE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OPERATING COST</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Land rent (42 rai × ฿/rai/yr)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Staff</t>
   </si>
   <si>
-    <t xml:space="preserve">Utilities</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Marketing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Admin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Maintenance</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CAPEX (one-time)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">20 pre-built farm-stay units (THB/unit)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Site infrastructure (roads, water, electrical backbone)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EV park-and-stay pad (THB/pad)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DC fast charger, incl. install (THB/charger)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Restaurant building + kitchen + furnishing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reception/admin building</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Equipment &amp; vehicles</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Working capital reserve</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Contingency + legal/permits/lease deposit</t>
-  </si>
-  <si>
-    <t xml:space="preserve">YEAR 5 — TERMINAL TRANSACTION (sell houses, buy land)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Farm-stay unit resale value (% of original cost)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Land purchase price at Year 5 (THB, total 42 rai)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Placeholder: ~2.3M/rai per the owner's earlier pricing — confirm the actual negotiated price</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rent credited toward purchase price (% of 5-yr rent paid)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A rent-to-own term worth negotiating with the owner</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rai gifted to the sanctuary after purchase</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Informational only — no cost impact here; the remaining rai stay with the tourism business</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Capital Expenditure</t>
-  </si>
-  <si>
-    <t xml:space="preserve">~฿ 38.0M upfront — no land purchase in this phase</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Item</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Amount (THB)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">% of total</t>
-  </si>
-  <si>
-    <t xml:space="preserve">20 pre-built farm-stay units</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10 EV park-and-stay pads</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5 DC fast chargers (incl. install)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOTAL CAPEX</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5-Year Operating Plan</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Farm-stay + EV park &amp; charging + restaurant, on leased land</t>
-  </si>
-  <si>
-    <t xml:space="preserve">REVENUE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Farm-stay (units × occ × rate × 365)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EV park &amp; stay (bays × occ × rate × 365)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fast charging (chargers × sessions/day × kWh × price × 365)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Restaurant (covers/day × avg spend × 365)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOTAL REVENUE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OPERATING COST</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Land rent (42 rai × ฿/rai/yr)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Food &amp; beverage cost of goods</t>
+    <t xml:space="preserve">Horse feed &amp; routine care</t>
   </si>
   <si>
     <t xml:space="preserve">Electricity resale cost (wholesale)</t>
@@ -667,23 +700,23 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="166" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="168" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -715,15 +748,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="13" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="166" fontId="13" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -918,9 +951,9 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>Capex!$B$6:$B$14</c:f>
+              <c:f>Capex!$B$6:$B$16</c:f>
               <c:strCache>
-                <c:ptCount val="9"/>
+                <c:ptCount val="11"/>
                 <c:pt idx="0">
                   <c:v>20 pre-built farm-stay units</c:v>
                 </c:pt>
@@ -934,18 +967,24 @@
                   <c:v>5 DC fast chargers (incl. install)</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>Restaurant building + kitchen + furnishing</c:v>
+                  <c:v>Horse stable barn (20 stalls) + tack/feed room</c:v>
                 </c:pt>
                 <c:pt idx="5">
+                  <c:v>Paddock &amp; perimeter fencing</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Initial stable fit-out &amp; onboarding</c:v>
+                </c:pt>
+                <c:pt idx="7">
                   <c:v>Reception/admin building</c:v>
                 </c:pt>
-                <c:pt idx="6">
+                <c:pt idx="8">
                   <c:v>Equipment &amp; vehicles</c:v>
                 </c:pt>
-                <c:pt idx="7">
+                <c:pt idx="9">
                   <c:v>Working capital reserve</c:v>
                 </c:pt>
-                <c:pt idx="8">
+                <c:pt idx="10">
                   <c:v>Contingency + legal/permits/lease deposit</c:v>
                 </c:pt>
               </c:strCache>
@@ -953,10 +992,10 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Capex!$C$6:$C$14</c:f>
+              <c:f>Capex!$C$6:$C$16</c:f>
               <c:numCache>
                 <c:formatCode>\฿#,##0;"(฿"#,##0\);\-</c:formatCode>
-                <c:ptCount val="9"/>
+                <c:ptCount val="11"/>
                 <c:pt idx="0">
                   <c:v>10000000</c:v>
                 </c:pt>
@@ -970,18 +1009,24 @@
                   <c:v>6000000</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>5000000</c:v>
+                  <c:v>11000000</c:v>
                 </c:pt>
                 <c:pt idx="5">
+                  <c:v>1500000</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>500000</c:v>
+                </c:pt>
+                <c:pt idx="7">
                   <c:v>2000000</c:v>
                 </c:pt>
-                <c:pt idx="6">
+                <c:pt idx="8">
                   <c:v>1500000</c:v>
                 </c:pt>
-                <c:pt idx="7">
+                <c:pt idx="9">
                   <c:v>1500000</c:v>
                 </c:pt>
-                <c:pt idx="8">
+                <c:pt idx="10">
                   <c:v>2000000</c:v>
                 </c:pt>
               </c:numCache>
@@ -990,11 +1035,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="74106501"/>
-        <c:axId val="55546696"/>
+        <c:axId val="51604556"/>
+        <c:axId val="31281034"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="74106501"/>
+        <c:axId val="51604556"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1026,7 +1071,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="55546696"/>
+        <c:crossAx val="31281034"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1034,7 +1079,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="55546696"/>
+        <c:axId val="31281034"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1076,7 +1121,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="74106501"/>
+        <c:crossAx val="51604556"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1221,24 +1266,24 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Operating P&amp;L'!$C$24:$G$24</c:f>
+              <c:f>'Operating P&amp;L'!$C$25:$G$25</c:f>
               <c:numCache>
                 <c:formatCode>\฿#,##0;"(฿"#,##0\);\-</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>8067700</c:v>
+                  <c:v>355500</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>14908125</c:v>
+                  <c:v>2363125</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>20630300</c:v>
+                  <c:v>3586500</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>22556875</c:v>
+                  <c:v>4262375</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>23437350</c:v>
+                  <c:v>4889700</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1253,11 +1298,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="1"/>
-        <c:axId val="2696513"/>
-        <c:axId val="69295974"/>
+        <c:axId val="91964386"/>
+        <c:axId val="562208"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="2696513"/>
+        <c:axId val="91964386"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1289,7 +1334,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="69295974"/>
+        <c:crossAx val="562208"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1297,7 +1342,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="69295974"/>
+        <c:axId val="562208"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1339,7 +1384,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="2696513"/>
+        <c:crossAx val="91964386"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1482,22 +1527,22 @@
                 <c:formatCode>\฿#,##0;"(฿"#,##0\);\-</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>-38000000</c:v>
+                  <c:v>-46000000</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>8067700</c:v>
+                  <c:v>355500</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>14908125</c:v>
+                  <c:v>2363125</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>20630300</c:v>
+                  <c:v>3586500</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>22556875</c:v>
+                  <c:v>4262375</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>-69162650</c:v>
+                  <c:v>-87710300</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1505,8 +1550,8 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="25984799"/>
-        <c:axId val="89793976"/>
+        <c:axId val="35122467"/>
+        <c:axId val="36506063"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -1592,22 +1637,22 @@
                 <c:formatCode>\฿#,##0;"(฿"#,##0\);\-</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>-38000000</c:v>
+                  <c:v>-46000000</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>-29932300</c:v>
+                  <c:v>-45644500</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>-15024175</c:v>
+                  <c:v>-43281375</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5606125</c:v>
+                  <c:v>-39694875</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>28163000</c:v>
+                  <c:v>-35432500</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>-40999650</c:v>
+                  <c:v>-123142800</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1622,11 +1667,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="1"/>
-        <c:axId val="25984799"/>
-        <c:axId val="89793976"/>
+        <c:axId val="35122467"/>
+        <c:axId val="36506063"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="25984799"/>
+        <c:axId val="35122467"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1658,7 +1703,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="89793976"/>
+        <c:crossAx val="36506063"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1666,7 +1711,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="89793976"/>
+        <c:axId val="36506063"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1742,7 +1787,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="25984799"/>
+        <c:crossAx val="35122467"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1885,22 +1930,22 @@
                 <c:formatCode>\฿#,##0;"(฿"#,##0\);\-</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>-38000000</c:v>
+                  <c:v>-46000000</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>8067700</c:v>
+                  <c:v>355500</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>14908125</c:v>
+                  <c:v>2363125</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>20630300</c:v>
+                  <c:v>3586500</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>22556875</c:v>
+                  <c:v>4262375</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>-69162650</c:v>
+                  <c:v>-87710300</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1908,8 +1953,8 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="91340746"/>
-        <c:axId val="13948899"/>
+        <c:axId val="26131556"/>
+        <c:axId val="30698197"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -1995,22 +2040,22 @@
                 <c:formatCode>\฿#,##0;"(฿"#,##0\);\-</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>-38000000</c:v>
+                  <c:v>-46000000</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>-29932300</c:v>
+                  <c:v>-45644500</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>-15024175</c:v>
+                  <c:v>-43281375</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5606125</c:v>
+                  <c:v>-39694875</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>28163000</c:v>
+                  <c:v>-35432500</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>-40999650</c:v>
+                  <c:v>-123142800</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2025,11 +2070,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="1"/>
-        <c:axId val="91340746"/>
-        <c:axId val="13948899"/>
+        <c:axId val="26131556"/>
+        <c:axId val="30698197"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="91340746"/>
+        <c:axId val="26131556"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2061,7 +2106,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="13948899"/>
+        <c:crossAx val="30698197"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2069,7 +2114,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="13948899"/>
+        <c:axId val="30698197"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2145,7 +2190,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="91340746"/>
+        <c:crossAx val="26131556"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2214,13 +2259,13 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>25</xdr:row>
+      <xdr:row>26</xdr:row>
       <xdr:rowOff>100800</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
       <xdr:colOff>692280</xdr:colOff>
-      <xdr:row>38</xdr:row>
+      <xdr:row>39</xdr:row>
       <xdr:rowOff>144000</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
@@ -2229,7 +2274,7 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="222120" y="4924440"/>
+        <a:off x="222120" y="5114880"/>
         <a:ext cx="5759640" cy="2519640"/>
       </xdr:xfrm>
       <a:graphic>
@@ -2493,7 +2538,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="B1:B24"/>
+  <dimension ref="B1:B26"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2.5"/>
@@ -2527,18 +2572,18 @@
         <v>4</v>
       </c>
     </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B9" s="3" t="s">
+        <v>5</v>
+      </c>
+    </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="4" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="3" t="s">
+      <c r="B10" s="3" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="3" t="s">
+      <c r="B12" s="4" t="s">
         <v>7</v>
       </c>
     </row>
@@ -2552,18 +2597,18 @@
         <v>9</v>
       </c>
     </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B15" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="4" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="3" t="s">
+      <c r="B16" s="3" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="3" t="s">
+      <c r="B18" s="4" t="s">
         <v>12</v>
       </c>
     </row>
@@ -2582,14 +2627,24 @@
         <v>15</v>
       </c>
     </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B22" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="3" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B24" s="3" t="s">
         <v>17</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B25" s="3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B26" s="3" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>
@@ -2608,7 +2663,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="B1:H59"/>
+  <dimension ref="B1:H62"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2.5"/>
@@ -2619,17 +2674,17 @@
     <row r="1" customFormat="false" ht="6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="2" customFormat="false" ht="22.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="2" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="5" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C5" s="5"/>
       <c r="D5" s="5"/>
@@ -2640,7 +2695,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C6" s="6" t="n">
         <v>42</v>
@@ -2648,18 +2703,18 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="3" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C7" s="7" t="n">
         <v>4000</v>
       </c>
       <c r="H7" s="8" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="3" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C8" s="9" t="n">
         <v>46296</v>
@@ -2667,7 +2722,7 @@
     </row>
     <row r="10" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B10" s="5" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C10" s="5"/>
       <c r="D10" s="5"/>
@@ -2678,7 +2733,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="3" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C11" s="6" t="n">
         <v>20</v>
@@ -2686,58 +2741,64 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="C12" s="10" t="n">
-        <v>2800</v>
+        <v>29</v>
+      </c>
+      <c r="C12" s="7" t="n">
+        <v>180000</v>
+      </c>
+      <c r="H12" s="8" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B13" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="C13" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="D13" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="E13" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="F13" s="11" t="s">
+      <c r="C13" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="G13" s="11" t="s">
+      <c r="D13" s="10" t="s">
         <v>33</v>
       </c>
+      <c r="E13" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="F13" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="G13" s="10" t="s">
+        <v>36</v>
+      </c>
       <c r="H13" s="4" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="C14" s="12" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="D14" s="12" t="n">
-        <v>0.45</v>
-      </c>
-      <c r="E14" s="12" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="F14" s="12" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="G14" s="12" t="n">
-        <v>0.62</v>
+        <v>38</v>
+      </c>
+      <c r="C14" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="D14" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="E14" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="F14" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="G14" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="H14" s="8" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B16" s="5" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C16" s="5"/>
       <c r="D16" s="5"/>
@@ -2748,7 +2809,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="3" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="C17" s="6" t="n">
         <v>10</v>
@@ -2756,38 +2817,38 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="C18" s="10" t="n">
+        <v>42</v>
+      </c>
+      <c r="C18" s="11" t="n">
         <v>900</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B19" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="C19" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="D19" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="E19" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="F19" s="11" t="s">
+      <c r="C19" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="G19" s="11" t="s">
+      <c r="D19" s="10" t="s">
         <v>33</v>
       </c>
+      <c r="E19" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="F19" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="G19" s="10" t="s">
+        <v>36</v>
+      </c>
       <c r="H19" s="4" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="3" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="C20" s="12" t="n">
         <v>0.2</v>
@@ -2807,7 +2868,7 @@
     </row>
     <row r="22" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B22" s="5" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="C22" s="5"/>
       <c r="D22" s="5"/>
@@ -2818,7 +2879,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="3" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="C23" s="6" t="n">
         <v>5</v>
@@ -2826,54 +2887,54 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="C24" s="10" t="n">
+        <v>46</v>
+      </c>
+      <c r="C24" s="11" t="n">
         <v>35</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="C25" s="10" t="n">
+        <v>47</v>
+      </c>
+      <c r="C25" s="11" t="n">
         <v>8</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="C26" s="10" t="n">
+        <v>48</v>
+      </c>
+      <c r="C26" s="11" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B27" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="C27" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="D27" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="E27" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="F27" s="11" t="s">
+      <c r="C27" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="G27" s="11" t="s">
+      <c r="D27" s="10" t="s">
         <v>33</v>
       </c>
+      <c r="E27" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="F27" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="G27" s="10" t="s">
+        <v>36</v>
+      </c>
       <c r="H27" s="4" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="3" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="C28" s="6" t="n">
         <v>4</v>
@@ -2893,7 +2954,7 @@
     </row>
     <row r="30" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B30" s="5" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="C30" s="5"/>
       <c r="D30" s="5"/>
@@ -2904,66 +2965,69 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="C31" s="10" t="n">
-        <v>350</v>
+        <v>51</v>
+      </c>
+      <c r="C31" s="7" t="n">
+        <v>15000</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="C32" s="13" t="n">
-        <v>0.32</v>
+        <v>52</v>
+      </c>
+      <c r="C32" s="11" t="n">
+        <v>4500</v>
+      </c>
+      <c r="H32" s="8" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B33" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="C33" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="D33" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="E33" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="F33" s="11" t="s">
+      <c r="C33" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="G33" s="11" t="s">
+      <c r="D33" s="10" t="s">
         <v>33</v>
       </c>
+      <c r="E33" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="F33" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="G33" s="10" t="s">
+        <v>36</v>
+      </c>
       <c r="H33" s="4" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="3" t="s">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="C34" s="6" t="n">
-        <v>60</v>
+        <v>15</v>
       </c>
       <c r="D34" s="6" t="n">
-        <v>100</v>
+        <v>20</v>
       </c>
       <c r="E34" s="6" t="n">
-        <v>140</v>
+        <v>20</v>
       </c>
       <c r="F34" s="6" t="n">
-        <v>150</v>
+        <v>20</v>
       </c>
       <c r="G34" s="6" t="n">
-        <v>155</v>
+        <v>20</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B36" s="5" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="C36" s="5"/>
       <c r="D36" s="5"/>
@@ -2974,260 +3038,296 @@
     </row>
     <row r="37" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B37" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="C37" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="D37" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="E37" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="F37" s="11" t="s">
+      <c r="C37" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="G37" s="11" t="s">
+      <c r="D37" s="10" t="s">
         <v>33</v>
       </c>
+      <c r="E37" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="F37" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="G37" s="10" t="s">
+        <v>36</v>
+      </c>
       <c r="H37" s="4" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="C38" s="10" t="n">
-        <v>2232000</v>
-      </c>
-      <c r="D38" s="10" t="n">
-        <v>2800000</v>
-      </c>
-      <c r="E38" s="10" t="n">
-        <v>3200000</v>
-      </c>
-      <c r="F38" s="10" t="n">
-        <v>3400000</v>
-      </c>
-      <c r="G38" s="10" t="n">
-        <v>3500000</v>
+        <v>56</v>
+      </c>
+      <c r="C38" s="11" t="n">
+        <v>1300000</v>
+      </c>
+      <c r="D38" s="11" t="n">
+        <v>1500000</v>
+      </c>
+      <c r="E38" s="11" t="n">
+        <v>1650000</v>
+      </c>
+      <c r="F38" s="11" t="n">
+        <v>1750000</v>
+      </c>
+      <c r="G38" s="11" t="n">
+        <v>1800000</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B39" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="C39" s="10" t="n">
-        <v>800000</v>
-      </c>
-      <c r="D39" s="10" t="n">
-        <v>950000</v>
-      </c>
-      <c r="E39" s="10" t="n">
-        <v>1100000</v>
-      </c>
-      <c r="F39" s="10" t="n">
-        <v>1150000</v>
-      </c>
-      <c r="G39" s="10" t="n">
-        <v>1200000</v>
+        <v>57</v>
+      </c>
+      <c r="C39" s="11" t="n">
+        <v>420000</v>
+      </c>
+      <c r="D39" s="11" t="n">
+        <v>480000</v>
+      </c>
+      <c r="E39" s="11" t="n">
+        <v>480000</v>
+      </c>
+      <c r="F39" s="11" t="n">
+        <v>480000</v>
+      </c>
+      <c r="G39" s="11" t="n">
+        <v>480000</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B40" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="C40" s="10" t="n">
-        <v>600000</v>
-      </c>
-      <c r="D40" s="10" t="n">
-        <v>500000</v>
-      </c>
-      <c r="E40" s="10" t="n">
-        <v>500000</v>
-      </c>
-      <c r="F40" s="10" t="n">
-        <v>500000</v>
-      </c>
-      <c r="G40" s="10" t="n">
-        <v>500000</v>
+        <v>58</v>
+      </c>
+      <c r="C40" s="11" t="n">
+        <v>650000</v>
+      </c>
+      <c r="D40" s="11" t="n">
+        <v>750000</v>
+      </c>
+      <c r="E40" s="11" t="n">
+        <v>850000</v>
+      </c>
+      <c r="F40" s="11" t="n">
+        <v>900000</v>
+      </c>
+      <c r="G40" s="11" t="n">
+        <v>950000</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B41" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="C41" s="10" t="n">
-        <v>400000</v>
-      </c>
-      <c r="D41" s="10" t="n">
-        <v>450000</v>
-      </c>
-      <c r="E41" s="10" t="n">
+        <v>59</v>
+      </c>
+      <c r="C41" s="11" t="n">
+        <v>600000</v>
+      </c>
+      <c r="D41" s="11" t="n">
         <v>500000</v>
       </c>
-      <c r="F41" s="10" t="n">
-        <v>520000</v>
-      </c>
-      <c r="G41" s="10" t="n">
-        <v>540000</v>
+      <c r="E41" s="11" t="n">
+        <v>500000</v>
+      </c>
+      <c r="F41" s="11" t="n">
+        <v>500000</v>
+      </c>
+      <c r="G41" s="11" t="n">
+        <v>500000</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B42" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="C42" s="10" t="n">
+        <v>60</v>
+      </c>
+      <c r="C42" s="11" t="n">
+        <v>400000</v>
+      </c>
+      <c r="D42" s="11" t="n">
+        <v>450000</v>
+      </c>
+      <c r="E42" s="11" t="n">
         <v>500000</v>
       </c>
-      <c r="D42" s="10" t="n">
+      <c r="F42" s="11" t="n">
+        <v>520000</v>
+      </c>
+      <c r="G42" s="11" t="n">
+        <v>540000</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B43" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C43" s="11" t="n">
+        <v>500000</v>
+      </c>
+      <c r="D43" s="11" t="n">
         <v>600000</v>
       </c>
-      <c r="E42" s="10" t="n">
+      <c r="E43" s="11" t="n">
         <v>700000</v>
       </c>
-      <c r="F42" s="10" t="n">
+      <c r="F43" s="11" t="n">
         <v>750000</v>
       </c>
-      <c r="G42" s="10" t="n">
+      <c r="G43" s="11" t="n">
         <v>800000</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B44" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="C44" s="5"/>
-      <c r="D44" s="5"/>
-      <c r="E44" s="5"/>
-      <c r="F44" s="5"/>
-      <c r="G44" s="5"/>
-      <c r="H44" s="5"/>
-    </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B45" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="C45" s="10" t="n">
-        <v>500000</v>
-      </c>
+    <row r="45" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B45" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="C45" s="5"/>
+      <c r="D45" s="5"/>
+      <c r="E45" s="5"/>
+      <c r="F45" s="5"/>
+      <c r="G45" s="5"/>
+      <c r="H45" s="5"/>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B46" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="C46" s="10" t="n">
-        <v>8000000</v>
+        <v>63</v>
+      </c>
+      <c r="C46" s="11" t="n">
+        <v>500000</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B47" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="C47" s="10" t="n">
-        <v>200000</v>
+        <v>64</v>
+      </c>
+      <c r="C47" s="11" t="n">
+        <v>8000000</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B48" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="C48" s="10" t="n">
-        <v>1200000</v>
+        <v>65</v>
+      </c>
+      <c r="C48" s="11" t="n">
+        <v>200000</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B49" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="C49" s="10" t="n">
-        <v>5000000</v>
+        <v>66</v>
+      </c>
+      <c r="C49" s="11" t="n">
+        <v>1200000</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B50" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="C50" s="10" t="n">
-        <v>2000000</v>
+        <v>67</v>
+      </c>
+      <c r="C50" s="11" t="n">
+        <v>11000000</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B51" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="C51" s="10" t="n">
+        <v>68</v>
+      </c>
+      <c r="C51" s="11" t="n">
         <v>1500000</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B52" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="C52" s="10" t="n">
-        <v>1500000</v>
+        <v>69</v>
+      </c>
+      <c r="C52" s="11" t="n">
+        <v>500000</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B53" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="C53" s="10" t="n">
+        <v>70</v>
+      </c>
+      <c r="C53" s="11" t="n">
         <v>2000000</v>
       </c>
     </row>
-    <row r="55" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B55" s="14" t="s">
-        <v>64</v>
-      </c>
-      <c r="C55" s="14"/>
-      <c r="D55" s="14"/>
-      <c r="E55" s="14"/>
-      <c r="F55" s="14"/>
-      <c r="G55" s="14"/>
-      <c r="H55" s="14"/>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B54" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="C54" s="11" t="n">
+        <v>1500000</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B55" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="C55" s="11" t="n">
+        <v>1500000</v>
+      </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B56" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="C56" s="12" t="n">
-        <v>0.4</v>
-      </c>
-    </row>
-    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B57" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="C57" s="7" t="n">
-        <v>96600000</v>
-      </c>
-      <c r="H57" s="8" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B58" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="C58" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="H58" s="8" t="s">
-        <v>69</v>
-      </c>
+        <v>73</v>
+      </c>
+      <c r="C56" s="11" t="n">
+        <v>2000000</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B58" s="13" t="s">
+        <v>74</v>
+      </c>
+      <c r="C58" s="13"/>
+      <c r="D58" s="13"/>
+      <c r="E58" s="13"/>
+      <c r="F58" s="13"/>
+      <c r="G58" s="13"/>
+      <c r="H58" s="13"/>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B59" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="C59" s="6" t="n">
+        <v>75</v>
+      </c>
+      <c r="C59" s="12" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B60" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="C60" s="7" t="n">
+        <v>96600000</v>
+      </c>
+      <c r="H60" s="8" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B61" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="C61" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H61" s="8" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B62" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="C62" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="H59" s="8" t="s">
-        <v>71</v>
+      <c r="H62" s="8" t="s">
+        <v>81</v>
       </c>
     </row>
   </sheetData>
@@ -3238,8 +3338,8 @@
     <mergeCell ref="B22:H22"/>
     <mergeCell ref="B30:H30"/>
     <mergeCell ref="B36:H36"/>
-    <mergeCell ref="B44:H44"/>
-    <mergeCell ref="B55:H55"/>
+    <mergeCell ref="B45:H45"/>
+    <mergeCell ref="B58:H58"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -3256,7 +3356,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="B1:D15"/>
+  <dimension ref="B1:D17"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2.5"/>
@@ -3267,151 +3367,177 @@
     <row r="1" customFormat="false" ht="6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="2" customFormat="false" ht="22.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="1" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="2" t="s">
-        <v>73</v>
+        <v>83</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="15" t="s">
-        <v>74</v>
+        <v>84</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="D5" s="15" t="s">
-        <v>76</v>
+        <v>86</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="3" t="s">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="C6" s="16" t="n">
-        <f aca="false">Assumptions!$C$45*Assumptions!$C$11</f>
+        <f aca="false">Assumptions!$C$46*Assumptions!$C$11</f>
         <v>10000000</v>
       </c>
       <c r="D6" s="17" t="n">
-        <f aca="false">C6/$C$15</f>
-        <v>0.263157894736842</v>
+        <f aca="false">C6/$C$17</f>
+        <v>0.217391304347826</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="3" t="s">
-        <v>56</v>
+        <v>64</v>
       </c>
       <c r="C7" s="16" t="n">
-        <f aca="false">Assumptions!$C$46</f>
+        <f aca="false">Assumptions!$C$47</f>
         <v>8000000</v>
       </c>
       <c r="D7" s="17" t="n">
-        <f aca="false">C7/$C$15</f>
-        <v>0.210526315789474</v>
+        <f aca="false">C7/$C$17</f>
+        <v>0.173913043478261</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="3" t="s">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="C8" s="16" t="n">
-        <f aca="false">Assumptions!$C$47*Assumptions!$C$17</f>
+        <f aca="false">Assumptions!$C$48*Assumptions!$C$17</f>
         <v>2000000</v>
       </c>
       <c r="D8" s="17" t="n">
-        <f aca="false">C8/$C$15</f>
-        <v>0.0526315789473684</v>
+        <f aca="false">C8/$C$17</f>
+        <v>0.0434782608695652</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="3" t="s">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="C9" s="16" t="n">
-        <f aca="false">Assumptions!$C$48*Assumptions!$C$23</f>
+        <f aca="false">Assumptions!$C$49*Assumptions!$C$23</f>
         <v>6000000</v>
       </c>
       <c r="D9" s="17" t="n">
-        <f aca="false">C9/$C$15</f>
-        <v>0.157894736842105</v>
+        <f aca="false">C9/$C$17</f>
+        <v>0.130434782608696</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="3" t="s">
-        <v>59</v>
+        <v>67</v>
       </c>
       <c r="C10" s="16" t="n">
-        <f aca="false">Assumptions!$C$49</f>
-        <v>5000000</v>
+        <f aca="false">Assumptions!$C$50</f>
+        <v>11000000</v>
       </c>
       <c r="D10" s="17" t="n">
-        <f aca="false">C10/$C$15</f>
-        <v>0.131578947368421</v>
+        <f aca="false">C10/$C$17</f>
+        <v>0.239130434782609</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="3" t="s">
-        <v>60</v>
+        <v>68</v>
       </c>
       <c r="C11" s="16" t="n">
-        <f aca="false">Assumptions!$C$50</f>
-        <v>2000000</v>
+        <f aca="false">Assumptions!$C$51</f>
+        <v>1500000</v>
       </c>
       <c r="D11" s="17" t="n">
-        <f aca="false">C11/$C$15</f>
-        <v>0.0526315789473684</v>
+        <f aca="false">C11/$C$17</f>
+        <v>0.0326086956521739</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="3" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="C12" s="16" t="n">
-        <f aca="false">Assumptions!$C$51</f>
-        <v>1500000</v>
+        <f aca="false">Assumptions!$C$52</f>
+        <v>500000</v>
       </c>
       <c r="D12" s="17" t="n">
-        <f aca="false">C12/$C$15</f>
-        <v>0.0394736842105263</v>
+        <f aca="false">C12/$C$17</f>
+        <v>0.0108695652173913</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="3" t="s">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="C13" s="16" t="n">
-        <f aca="false">Assumptions!$C$52</f>
-        <v>1500000</v>
+        <f aca="false">Assumptions!$C$53</f>
+        <v>2000000</v>
       </c>
       <c r="D13" s="17" t="n">
-        <f aca="false">C13/$C$15</f>
-        <v>0.0394736842105263</v>
+        <f aca="false">C13/$C$17</f>
+        <v>0.0434782608695652</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="3" t="s">
-        <v>63</v>
+        <v>71</v>
       </c>
       <c r="C14" s="16" t="n">
-        <f aca="false">Assumptions!$C$53</f>
+        <f aca="false">Assumptions!$C$54</f>
+        <v>1500000</v>
+      </c>
+      <c r="D14" s="17" t="n">
+        <f aca="false">C14/$C$17</f>
+        <v>0.0326086956521739</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B15" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="C15" s="16" t="n">
+        <f aca="false">Assumptions!$C$55</f>
+        <v>1500000</v>
+      </c>
+      <c r="D15" s="17" t="n">
+        <f aca="false">C15/$C$17</f>
+        <v>0.0326086956521739</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B16" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="C16" s="16" t="n">
+        <f aca="false">Assumptions!$C$56</f>
         <v>2000000</v>
       </c>
-      <c r="D14" s="17" t="n">
-        <f aca="false">C14/$C$15</f>
-        <v>0.0526315789473684</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="18" t="s">
-        <v>80</v>
-      </c>
-      <c r="C15" s="19" t="n">
-        <f aca="false">SUM(C6:C14)</f>
-        <v>38000000</v>
-      </c>
-      <c r="D15" s="20" t="n">
+      <c r="D16" s="17" t="n">
+        <f aca="false">C16/$C$17</f>
+        <v>0.0434782608695652</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B17" s="18" t="s">
+        <v>90</v>
+      </c>
+      <c r="C17" s="19" t="n">
+        <f aca="false">SUM(C6:C16)</f>
+        <v>46000000</v>
+      </c>
+      <c r="D17" s="20" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3432,7 +3558,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="B1:H24"/>
+  <dimension ref="B1:H25"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2.5"/>
@@ -3443,40 +3569,40 @@
     <row r="1" customFormat="false" ht="6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="2" customFormat="false" ht="22.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="1" t="s">
-        <v>81</v>
+        <v>91</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="2" t="s">
-        <v>82</v>
+        <v>92</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="C5" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="D5" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="E5" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="F5" s="11" t="s">
+      <c r="C5" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="G5" s="11" t="s">
+      <c r="D5" s="10" t="s">
         <v>33</v>
       </c>
+      <c r="E5" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="F5" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="G5" s="10" t="s">
+        <v>36</v>
+      </c>
       <c r="H5" s="4" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B6" s="5" t="s">
-        <v>83</v>
+        <v>93</v>
       </c>
       <c r="C6" s="5"/>
       <c r="D6" s="5"/>
@@ -3487,32 +3613,32 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="21" t="s">
-        <v>84</v>
+        <v>94</v>
       </c>
       <c r="C7" s="16" t="n">
-        <f aca="false">Assumptions!$C$11*Assumptions!$C$14*Assumptions!$C$12*365</f>
-        <v>6132000</v>
+        <f aca="false">Assumptions!$C$14*Assumptions!$C$12</f>
+        <v>1080000</v>
       </c>
       <c r="D7" s="16" t="n">
-        <f aca="false">Assumptions!$C$11*Assumptions!$D$14*Assumptions!$C$12*365</f>
-        <v>9198000</v>
+        <f aca="false">Assumptions!$D$14*Assumptions!$C$12</f>
+        <v>1800000</v>
       </c>
       <c r="E7" s="16" t="n">
-        <f aca="false">Assumptions!$C$11*Assumptions!$E$14*Assumptions!$C$12*365</f>
-        <v>11242000</v>
+        <f aca="false">Assumptions!$E$14*Assumptions!$C$12</f>
+        <v>2520000</v>
       </c>
       <c r="F7" s="16" t="n">
-        <f aca="false">Assumptions!$C$11*Assumptions!$F$14*Assumptions!$C$12*365</f>
-        <v>12264000</v>
+        <f aca="false">Assumptions!$F$14*Assumptions!$C$12</f>
+        <v>3060000</v>
       </c>
       <c r="G7" s="16" t="n">
-        <f aca="false">Assumptions!$C$11*Assumptions!$G$14*Assumptions!$C$12*365</f>
-        <v>12672800</v>
+        <f aca="false">Assumptions!$G$14*Assumptions!$C$12</f>
+        <v>3600000</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="21" t="s">
-        <v>85</v>
+        <v>95</v>
       </c>
       <c r="C8" s="16" t="n">
         <f aca="false">Assumptions!$C$17*Assumptions!$C$20*Assumptions!$C$18*365</f>
@@ -3537,7 +3663,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="21" t="s">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="C9" s="16" t="n">
         <f aca="false">Assumptions!$C$23*Assumptions!$C$28*Assumptions!$C$24*Assumptions!$C$25*365</f>
@@ -3562,57 +3688,57 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="21" t="s">
-        <v>87</v>
+        <v>97</v>
       </c>
       <c r="C10" s="16" t="n">
-        <f aca="false">Assumptions!$C$34*Assumptions!$C$31*365</f>
-        <v>7665000</v>
+        <f aca="false">Assumptions!$C$34*Assumptions!$C$31*12</f>
+        <v>2700000</v>
       </c>
       <c r="D10" s="16" t="n">
-        <f aca="false">Assumptions!$D$34*Assumptions!$C$31*365</f>
-        <v>12775000</v>
+        <f aca="false">Assumptions!$D$34*Assumptions!$C$31*12</f>
+        <v>3600000</v>
       </c>
       <c r="E10" s="16" t="n">
-        <f aca="false">Assumptions!$E$34*Assumptions!$C$31*365</f>
-        <v>17885000</v>
+        <f aca="false">Assumptions!$E$34*Assumptions!$C$31*12</f>
+        <v>3600000</v>
       </c>
       <c r="F10" s="16" t="n">
-        <f aca="false">Assumptions!$F$34*Assumptions!$C$31*365</f>
-        <v>19162500</v>
+        <f aca="false">Assumptions!$F$34*Assumptions!$C$31*12</f>
+        <v>3600000</v>
       </c>
       <c r="G10" s="16" t="n">
-        <f aca="false">Assumptions!$G$34*Assumptions!$C$31*365</f>
-        <v>19801250</v>
+        <f aca="false">Assumptions!$G$34*Assumptions!$C$31*12</f>
+        <v>3600000</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="18" t="s">
-        <v>88</v>
+        <v>98</v>
       </c>
       <c r="C11" s="19" t="n">
         <f aca="false">SUM(C7:C10)</f>
-        <v>16498000</v>
+        <v>6481000</v>
       </c>
       <c r="D11" s="19" t="n">
         <f aca="false">SUM(D7:D10)</f>
-        <v>26699750</v>
+        <v>10126750</v>
       </c>
       <c r="E11" s="19" t="n">
         <f aca="false">SUM(E7:E10)</f>
-        <v>35715250</v>
+        <v>12708250</v>
       </c>
       <c r="F11" s="19" t="n">
         <f aca="false">SUM(F7:F10)</f>
-        <v>38690000</v>
+        <v>13923500</v>
       </c>
       <c r="G11" s="19" t="n">
         <f aca="false">SUM(G7:G10)</f>
-        <v>40314250</v>
+        <v>15040200</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B13" s="5" t="s">
-        <v>89</v>
+        <v>99</v>
       </c>
       <c r="C13" s="5"/>
       <c r="D13" s="5"/>
@@ -3623,7 +3749,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="21" t="s">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="C14" s="16" t="n">
         <f aca="false">Assumptions!$C$6*Assumptions!$C$7</f>
@@ -3648,140 +3774,143 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="21" t="s">
-        <v>49</v>
+        <v>101</v>
       </c>
       <c r="C15" s="16" t="n">
         <f aca="false">Assumptions!$C$38</f>
-        <v>2232000</v>
+        <v>1300000</v>
       </c>
       <c r="D15" s="16" t="n">
         <f aca="false">Assumptions!$D$38</f>
-        <v>2800000</v>
+        <v>1500000</v>
       </c>
       <c r="E15" s="16" t="n">
         <f aca="false">Assumptions!$E$38</f>
-        <v>3200000</v>
+        <v>1650000</v>
       </c>
       <c r="F15" s="16" t="n">
         <f aca="false">Assumptions!$F$38</f>
-        <v>3400000</v>
+        <v>1750000</v>
       </c>
       <c r="G15" s="16" t="n">
         <f aca="false">Assumptions!$G$38</f>
-        <v>3500000</v>
+        <v>1800000</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="C16" s="22" t="n">
-        <f aca="false">C10*Assumptions!$C$32</f>
-        <v>2452800</v>
-      </c>
-      <c r="D16" s="22" t="n">
-        <f aca="false">D10*Assumptions!$C$32</f>
-        <v>4088000</v>
-      </c>
-      <c r="E16" s="22" t="n">
-        <f aca="false">E10*Assumptions!$C$32</f>
-        <v>5723200</v>
-      </c>
-      <c r="F16" s="22" t="n">
-        <f aca="false">F10*Assumptions!$C$32</f>
-        <v>6132000</v>
-      </c>
-      <c r="G16" s="22" t="n">
-        <f aca="false">G10*Assumptions!$C$32</f>
-        <v>6336400</v>
+      <c r="B16" s="21" t="s">
+        <v>57</v>
+      </c>
+      <c r="C16" s="16" t="n">
+        <f aca="false">Assumptions!$C$39</f>
+        <v>420000</v>
+      </c>
+      <c r="D16" s="16" t="n">
+        <f aca="false">Assumptions!$D$39</f>
+        <v>480000</v>
+      </c>
+      <c r="E16" s="16" t="n">
+        <f aca="false">Assumptions!$E$39</f>
+        <v>480000</v>
+      </c>
+      <c r="F16" s="16" t="n">
+        <f aca="false">Assumptions!$F$39</f>
+        <v>480000</v>
+      </c>
+      <c r="G16" s="16" t="n">
+        <f aca="false">Assumptions!$G$39</f>
+        <v>480000</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="21" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="C17" s="16" t="n">
+        <f aca="false">Assumptions!$C$34*Assumptions!$C$32*12</f>
+        <v>810000</v>
+      </c>
+      <c r="D17" s="16" t="n">
+        <f aca="false">Assumptions!$D$34*Assumptions!$C$32*12</f>
+        <v>1080000</v>
+      </c>
+      <c r="E17" s="16" t="n">
+        <f aca="false">Assumptions!$E$34*Assumptions!$C$32*12</f>
+        <v>1080000</v>
+      </c>
+      <c r="F17" s="16" t="n">
+        <f aca="false">Assumptions!$F$34*Assumptions!$C$32*12</f>
+        <v>1080000</v>
+      </c>
+      <c r="G17" s="16" t="n">
+        <f aca="false">Assumptions!$G$34*Assumptions!$C$32*12</f>
+        <v>1080000</v>
+      </c>
+      <c r="H17" s="8" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B18" s="21" t="s">
+        <v>103</v>
+      </c>
+      <c r="C18" s="16" t="n">
         <f aca="false">Assumptions!$C$23*Assumptions!$C$28*Assumptions!$C$24*365*Assumptions!$C$26</f>
         <v>1277500</v>
       </c>
-      <c r="D17" s="16" t="n">
+      <c r="D18" s="16" t="n">
         <f aca="false">Assumptions!$C$23*Assumptions!$D$28*Assumptions!$C$24*365*Assumptions!$C$26</f>
         <v>2235625</v>
       </c>
-      <c r="E17" s="16" t="n">
+      <c r="E18" s="16" t="n">
         <f aca="false">Assumptions!$C$23*Assumptions!$E$28*Assumptions!$C$24*365*Assumptions!$C$26</f>
         <v>3193750</v>
       </c>
-      <c r="F17" s="16" t="n">
+      <c r="F18" s="16" t="n">
         <f aca="false">Assumptions!$C$23*Assumptions!$F$28*Assumptions!$C$24*365*Assumptions!$C$26</f>
         <v>3513125</v>
       </c>
-      <c r="G17" s="16" t="n">
+      <c r="G18" s="16" t="n">
         <f aca="false">Assumptions!$C$23*Assumptions!$G$28*Assumptions!$C$24*365*Assumptions!$C$26</f>
         <v>3832500</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="21" t="s">
-        <v>50</v>
-      </c>
-      <c r="C18" s="16" t="n">
-        <f aca="false">Assumptions!$C$39</f>
-        <v>800000</v>
-      </c>
-      <c r="D18" s="16" t="n">
-        <f aca="false">Assumptions!$D$39</f>
-        <v>950000</v>
-      </c>
-      <c r="E18" s="16" t="n">
-        <f aca="false">Assumptions!$E$39</f>
-        <v>1100000</v>
-      </c>
-      <c r="F18" s="16" t="n">
-        <f aca="false">Assumptions!$F$39</f>
-        <v>1150000</v>
-      </c>
-      <c r="G18" s="16" t="n">
-        <f aca="false">Assumptions!$G$39</f>
-        <v>1200000</v>
-      </c>
-    </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="21" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="C19" s="16" t="n">
         <f aca="false">Assumptions!$C$40</f>
-        <v>600000</v>
+        <v>650000</v>
       </c>
       <c r="D19" s="16" t="n">
         <f aca="false">Assumptions!$D$40</f>
-        <v>500000</v>
+        <v>750000</v>
       </c>
       <c r="E19" s="16" t="n">
         <f aca="false">Assumptions!$E$40</f>
-        <v>500000</v>
+        <v>850000</v>
       </c>
       <c r="F19" s="16" t="n">
         <f aca="false">Assumptions!$F$40</f>
-        <v>500000</v>
+        <v>900000</v>
       </c>
       <c r="G19" s="16" t="n">
         <f aca="false">Assumptions!$G$40</f>
-        <v>500000</v>
+        <v>950000</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="21" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="C20" s="16" t="n">
         <f aca="false">Assumptions!$C$41</f>
-        <v>400000</v>
+        <v>600000</v>
       </c>
       <c r="D20" s="16" t="n">
         <f aca="false">Assumptions!$D$41</f>
-        <v>450000</v>
+        <v>500000</v>
       </c>
       <c r="E20" s="16" t="n">
         <f aca="false">Assumptions!$E$41</f>
@@ -3789,86 +3918,111 @@
       </c>
       <c r="F20" s="16" t="n">
         <f aca="false">Assumptions!$F$41</f>
-        <v>520000</v>
+        <v>500000</v>
       </c>
       <c r="G20" s="16" t="n">
         <f aca="false">Assumptions!$G$41</f>
-        <v>540000</v>
+        <v>500000</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="21" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="C21" s="16" t="n">
         <f aca="false">Assumptions!$C$42</f>
-        <v>500000</v>
+        <v>400000</v>
       </c>
       <c r="D21" s="16" t="n">
         <f aca="false">Assumptions!$D$42</f>
-        <v>600000</v>
+        <v>450000</v>
       </c>
       <c r="E21" s="16" t="n">
         <f aca="false">Assumptions!$E$42</f>
-        <v>700000</v>
+        <v>500000</v>
       </c>
       <c r="F21" s="16" t="n">
         <f aca="false">Assumptions!$F$42</f>
-        <v>750000</v>
+        <v>520000</v>
       </c>
       <c r="G21" s="16" t="n">
         <f aca="false">Assumptions!$G$42</f>
+        <v>540000</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B22" s="21" t="s">
+        <v>61</v>
+      </c>
+      <c r="C22" s="16" t="n">
+        <f aca="false">Assumptions!$C$43</f>
+        <v>500000</v>
+      </c>
+      <c r="D22" s="16" t="n">
+        <f aca="false">Assumptions!$D$43</f>
+        <v>600000</v>
+      </c>
+      <c r="E22" s="16" t="n">
+        <f aca="false">Assumptions!$E$43</f>
+        <v>700000</v>
+      </c>
+      <c r="F22" s="16" t="n">
+        <f aca="false">Assumptions!$F$43</f>
+        <v>750000</v>
+      </c>
+      <c r="G22" s="16" t="n">
+        <f aca="false">Assumptions!$G$43</f>
         <v>800000</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B22" s="18" t="s">
-        <v>93</v>
-      </c>
-      <c r="C22" s="19" t="n">
-        <f aca="false">SUM(C14:C21)</f>
-        <v>8430300</v>
-      </c>
-      <c r="D22" s="19" t="n">
-        <f aca="false">SUM(D14:D21)</f>
-        <v>11791625</v>
-      </c>
-      <c r="E22" s="19" t="n">
-        <f aca="false">SUM(E14:E21)</f>
-        <v>15084950</v>
-      </c>
-      <c r="F22" s="19" t="n">
-        <f aca="false">SUM(F14:F21)</f>
-        <v>16133125</v>
-      </c>
-      <c r="G22" s="19" t="n">
-        <f aca="false">SUM(G14:G21)</f>
-        <v>16876900</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B24" s="23" t="s">
-        <v>94</v>
-      </c>
-      <c r="C24" s="24" t="n">
-        <f aca="false">C11-C22</f>
-        <v>8067700</v>
-      </c>
-      <c r="D24" s="24" t="n">
-        <f aca="false">D11-D22</f>
-        <v>14908125</v>
-      </c>
-      <c r="E24" s="24" t="n">
-        <f aca="false">E11-E22</f>
-        <v>20630300</v>
-      </c>
-      <c r="F24" s="24" t="n">
-        <f aca="false">F11-F22</f>
-        <v>22556875</v>
-      </c>
-      <c r="G24" s="24" t="n">
-        <f aca="false">G11-G22</f>
-        <v>23437350</v>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B23" s="18" t="s">
+        <v>104</v>
+      </c>
+      <c r="C23" s="19" t="n">
+        <f aca="false">SUM(C14:C22)</f>
+        <v>6125500</v>
+      </c>
+      <c r="D23" s="19" t="n">
+        <f aca="false">SUM(D14:D22)</f>
+        <v>7763625</v>
+      </c>
+      <c r="E23" s="19" t="n">
+        <f aca="false">SUM(E14:E22)</f>
+        <v>9121750</v>
+      </c>
+      <c r="F23" s="19" t="n">
+        <f aca="false">SUM(F14:F22)</f>
+        <v>9661125</v>
+      </c>
+      <c r="G23" s="19" t="n">
+        <f aca="false">SUM(G14:G22)</f>
+        <v>10150500</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B25" s="22" t="s">
+        <v>105</v>
+      </c>
+      <c r="C25" s="23" t="n">
+        <f aca="false">C11-C23</f>
+        <v>355500</v>
+      </c>
+      <c r="D25" s="23" t="n">
+        <f aca="false">D11-D23</f>
+        <v>2363125</v>
+      </c>
+      <c r="E25" s="23" t="n">
+        <f aca="false">E11-E23</f>
+        <v>3586500</v>
+      </c>
+      <c r="F25" s="23" t="n">
+        <f aca="false">F11-F23</f>
+        <v>4262375</v>
+      </c>
+      <c r="G25" s="23" t="n">
+        <f aca="false">G11-G23</f>
+        <v>4889700</v>
       </c>
     </row>
   </sheetData>
@@ -3903,201 +4057,201 @@
     <row r="1" customFormat="false" ht="6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="2" customFormat="false" ht="22.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="1" t="s">
-        <v>95</v>
+        <v>106</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="2" t="s">
-        <v>96</v>
+        <v>107</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="4" t="s">
-        <v>97</v>
-      </c>
-      <c r="C5" s="11" t="s">
-        <v>98</v>
-      </c>
-      <c r="D5" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="E5" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="F5" s="11" t="s">
-        <v>31</v>
-      </c>
-      <c r="G5" s="11" t="s">
+        <v>108</v>
+      </c>
+      <c r="C5" s="10" t="s">
+        <v>109</v>
+      </c>
+      <c r="D5" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="H5" s="11" t="s">
+      <c r="E5" s="10" t="s">
         <v>33</v>
+      </c>
+      <c r="F5" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="G5" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="H5" s="10" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="3" t="s">
-        <v>99</v>
+        <v>110</v>
       </c>
       <c r="C6" s="16" t="n">
-        <f aca="false">-Capex!C15</f>
-        <v>-38000000</v>
-      </c>
-      <c r="D6" s="22" t="n">
+        <f aca="false">-Capex!C17</f>
+        <v>-46000000</v>
+      </c>
+      <c r="D6" s="24" t="n">
         <v>0</v>
       </c>
-      <c r="E6" s="22" t="n">
+      <c r="E6" s="24" t="n">
         <v>0</v>
       </c>
-      <c r="F6" s="22" t="n">
+      <c r="F6" s="24" t="n">
         <v>0</v>
       </c>
-      <c r="G6" s="22" t="n">
+      <c r="G6" s="24" t="n">
         <v>0</v>
       </c>
-      <c r="H6" s="22" t="n">
+      <c r="H6" s="24" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="3" t="s">
-        <v>100</v>
-      </c>
-      <c r="C7" s="22" t="n">
+        <v>111</v>
+      </c>
+      <c r="C7" s="24" t="n">
         <v>0</v>
       </c>
       <c r="D7" s="16" t="n">
-        <f aca="false">'Operating P&amp;L'!C24</f>
-        <v>8067700</v>
+        <f aca="false">'Operating P&amp;L'!C25</f>
+        <v>355500</v>
       </c>
       <c r="E7" s="16" t="n">
-        <f aca="false">'Operating P&amp;L'!D24</f>
-        <v>14908125</v>
+        <f aca="false">'Operating P&amp;L'!D25</f>
+        <v>2363125</v>
       </c>
       <c r="F7" s="16" t="n">
-        <f aca="false">'Operating P&amp;L'!E24</f>
-        <v>20630300</v>
+        <f aca="false">'Operating P&amp;L'!E25</f>
+        <v>3586500</v>
       </c>
       <c r="G7" s="16" t="n">
-        <f aca="false">'Operating P&amp;L'!F24</f>
-        <v>22556875</v>
+        <f aca="false">'Operating P&amp;L'!F25</f>
+        <v>4262375</v>
       </c>
       <c r="H7" s="16" t="n">
-        <f aca="false">'Operating P&amp;L'!G24</f>
-        <v>23437350</v>
+        <f aca="false">'Operating P&amp;L'!G25</f>
+        <v>4889700</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="C8" s="22" t="n">
+        <v>112</v>
+      </c>
+      <c r="C8" s="24" t="n">
         <v>0</v>
       </c>
-      <c r="D8" s="22" t="n">
+      <c r="D8" s="24" t="n">
         <v>0</v>
       </c>
-      <c r="E8" s="22" t="n">
+      <c r="E8" s="24" t="n">
         <v>0</v>
       </c>
-      <c r="F8" s="22" t="n">
+      <c r="F8" s="24" t="n">
         <v>0</v>
       </c>
-      <c r="G8" s="22" t="n">
+      <c r="G8" s="24" t="n">
         <v>0</v>
       </c>
       <c r="H8" s="25" t="n">
-        <f aca="false">-Assumptions!$C$57+((Assumptions!$C$45*Assumptions!$C$11)*Assumptions!$C$56)+((Assumptions!$C$6*Assumptions!$C$7*5)*Assumptions!$C$58)</f>
+        <f aca="false">-Assumptions!$C$60+((Assumptions!$C$46*Assumptions!$C$11)*Assumptions!$C$59)+((Assumptions!$C$6*Assumptions!$C$7*5)*Assumptions!$C$61)</f>
         <v>-92600000</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="26" t="s">
-        <v>102</v>
+        <v>113</v>
       </c>
       <c r="H9" s="27" t="n">
-        <f aca="false">+(Assumptions!$C$45*Assumptions!$C$11)*Assumptions!$C$56</f>
+        <f aca="false">+(Assumptions!$C$46*Assumptions!$C$11)*Assumptions!$C$59</f>
         <v>4000000</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="26" t="s">
-        <v>103</v>
+        <v>114</v>
       </c>
       <c r="H10" s="27" t="n">
-        <f aca="false">+(Assumptions!$C$6*Assumptions!$C$7*5)*Assumptions!$C$58</f>
+        <f aca="false">+(Assumptions!$C$6*Assumptions!$C$7*5)*Assumptions!$C$61</f>
         <v>0</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="26" t="s">
-        <v>104</v>
+        <v>115</v>
       </c>
       <c r="H11" s="28" t="n">
-        <f aca="false">-Assumptions!$C$57</f>
+        <f aca="false">-Assumptions!$C$60</f>
         <v>-96600000</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="18" t="s">
-        <v>105</v>
+        <v>116</v>
       </c>
       <c r="C13" s="19" t="n">
         <f aca="false">C6+C7</f>
-        <v>-38000000</v>
+        <v>-46000000</v>
       </c>
       <c r="D13" s="19" t="n">
         <f aca="false">D6+D7</f>
-        <v>8067700</v>
+        <v>355500</v>
       </c>
       <c r="E13" s="19" t="n">
         <f aca="false">E6+E7</f>
-        <v>14908125</v>
+        <v>2363125</v>
       </c>
       <c r="F13" s="19" t="n">
         <f aca="false">F6+F7</f>
-        <v>20630300</v>
+        <v>3586500</v>
       </c>
       <c r="G13" s="19" t="n">
         <f aca="false">G6+G7</f>
-        <v>22556875</v>
+        <v>4262375</v>
       </c>
       <c r="H13" s="19" t="n">
         <f aca="false">H6+H7+H8</f>
-        <v>-69162650</v>
+        <v>-87710300</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="23" t="s">
-        <v>106</v>
-      </c>
-      <c r="C14" s="24" t="n">
+      <c r="B14" s="22" t="s">
+        <v>117</v>
+      </c>
+      <c r="C14" s="23" t="n">
         <f aca="false">C13</f>
-        <v>-38000000</v>
-      </c>
-      <c r="D14" s="24" t="n">
+        <v>-46000000</v>
+      </c>
+      <c r="D14" s="23" t="n">
         <f aca="false">C14+D13</f>
-        <v>-29932300</v>
-      </c>
-      <c r="E14" s="24" t="n">
+        <v>-45644500</v>
+      </c>
+      <c r="E14" s="23" t="n">
         <f aca="false">D14+E13</f>
-        <v>-15024175</v>
-      </c>
-      <c r="F14" s="24" t="n">
+        <v>-43281375</v>
+      </c>
+      <c r="F14" s="23" t="n">
         <f aca="false">E14+F13</f>
-        <v>5606125</v>
-      </c>
-      <c r="G14" s="24" t="n">
+        <v>-39694875</v>
+      </c>
+      <c r="G14" s="23" t="n">
         <f aca="false">F14+G13</f>
-        <v>28163000</v>
-      </c>
-      <c r="H14" s="24" t="n">
+        <v>-35432500</v>
+      </c>
+      <c r="H14" s="23" t="n">
         <f aca="false">G14+H13</f>
-        <v>-40999650</v>
+        <v>-123142800</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B16" s="29" t="s">
-        <v>107</v>
+        <v>118</v>
       </c>
       <c r="C16" s="29"/>
       <c r="D16" s="29"/>
@@ -4136,17 +4290,17 @@
     <row r="1" customFormat="false" ht="6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="2" customFormat="false" ht="22.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="1" t="s">
-        <v>108</v>
+        <v>119</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="2" t="s">
-        <v>109</v>
+        <v>120</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B6" s="5" t="s">
-        <v>110</v>
+        <v>121</v>
       </c>
       <c r="C6" s="5"/>
       <c r="D6" s="5"/>
@@ -4157,24 +4311,24 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="3" t="s">
-        <v>111</v>
+        <v>122</v>
       </c>
       <c r="C7" s="30" t="s">
-        <v>112</v>
+        <v>123</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="3" t="s">
-        <v>113</v>
+        <v>124</v>
       </c>
       <c r="C8" s="16" t="n">
-        <f aca="false">Capex!C15</f>
-        <v>38000000</v>
+        <f aca="false">Capex!C17</f>
+        <v>46000000</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="3" t="s">
-        <v>114</v>
+        <v>125</v>
       </c>
       <c r="C9" s="16" t="n">
         <f aca="false">Assumptions!$C$6*Assumptions!$C$7</f>
@@ -4183,79 +4337,79 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="3" t="s">
-        <v>115</v>
+        <v>126</v>
       </c>
       <c r="C10" s="16" t="n">
-        <f aca="false">'Operating P&amp;L'!C24</f>
-        <v>8067700</v>
+        <f aca="false">'Operating P&amp;L'!C25</f>
+        <v>355500</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="3" t="s">
-        <v>116</v>
+        <v>127</v>
       </c>
       <c r="C11" s="16" t="n">
-        <f aca="false">'Operating P&amp;L'!G24</f>
-        <v>23437350</v>
+        <f aca="false">'Operating P&amp;L'!G25</f>
+        <v>4889700</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="3" t="s">
-        <v>117</v>
+        <v>128</v>
       </c>
       <c r="C12" s="16" t="n">
-        <f aca="false">SUM('Operating P&amp;L'!C24:G24)</f>
-        <v>89600350</v>
+        <f aca="false">SUM('Operating P&amp;L'!C25:G25)</f>
+        <v>15457200</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="3" t="s">
-        <v>118</v>
+        <v>129</v>
       </c>
       <c r="C13" s="16" t="n">
-        <f aca="false">Assumptions!$C$57</f>
+        <f aca="false">Assumptions!$C$60</f>
         <v>96600000</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="3" t="s">
-        <v>119</v>
+        <v>130</v>
       </c>
       <c r="C14" s="16" t="n">
-        <f aca="false">Assumptions!$C$45*Assumptions!$C$11*Assumptions!$C$56</f>
+        <f aca="false">Assumptions!$C$46*Assumptions!$C$11*Assumptions!$C$59</f>
         <v>4000000</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="3" t="s">
-        <v>120</v>
+        <v>131</v>
       </c>
       <c r="C15" s="16" t="n">
         <f aca="false">'Cash Flow'!H14</f>
-        <v>-40999650</v>
+        <v>-123142800</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="3" t="s">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="C16" s="31" t="n">
-        <f aca="false">Assumptions!$C$59</f>
+        <f aca="false">Assumptions!$C$62</f>
         <v>12</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="3" t="s">
-        <v>121</v>
+        <v>132</v>
       </c>
       <c r="C17" s="31" t="n">
-        <f aca="false">Assumptions!$C$6-Assumptions!$C$59</f>
+        <f aca="false">Assumptions!$C$6-Assumptions!$C$62</f>
         <v>30</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B19" s="5" t="s">
-        <v>122</v>
+        <v>133</v>
       </c>
       <c r="C19" s="5"/>
       <c r="D19" s="5"/>
@@ -4266,7 +4420,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="4" t="s">
-        <v>97</v>
+        <v>108</v>
       </c>
       <c r="C20" s="32" t="str">
         <f aca="false">'Cash Flow'!C5</f>
@@ -4295,65 +4449,65 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="3" t="s">
-        <v>105</v>
+        <v>116</v>
       </c>
       <c r="C21" s="16" t="n">
         <f aca="false">'Cash Flow'!C13</f>
-        <v>-38000000</v>
+        <v>-46000000</v>
       </c>
       <c r="D21" s="16" t="n">
         <f aca="false">'Cash Flow'!D13</f>
-        <v>8067700</v>
+        <v>355500</v>
       </c>
       <c r="E21" s="16" t="n">
         <f aca="false">'Cash Flow'!E13</f>
-        <v>14908125</v>
+        <v>2363125</v>
       </c>
       <c r="F21" s="16" t="n">
         <f aca="false">'Cash Flow'!F13</f>
-        <v>20630300</v>
+        <v>3586500</v>
       </c>
       <c r="G21" s="16" t="n">
         <f aca="false">'Cash Flow'!G13</f>
-        <v>22556875</v>
+        <v>4262375</v>
       </c>
       <c r="H21" s="16" t="n">
         <f aca="false">'Cash Flow'!H13</f>
-        <v>-69162650</v>
+        <v>-87710300</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="4" t="s">
-        <v>106</v>
+        <v>117</v>
       </c>
       <c r="C22" s="16" t="n">
         <f aca="false">'Cash Flow'!C14</f>
-        <v>-38000000</v>
+        <v>-46000000</v>
       </c>
       <c r="D22" s="16" t="n">
         <f aca="false">'Cash Flow'!D14</f>
-        <v>-29932300</v>
+        <v>-45644500</v>
       </c>
       <c r="E22" s="16" t="n">
         <f aca="false">'Cash Flow'!E14</f>
-        <v>-15024175</v>
+        <v>-43281375</v>
       </c>
       <c r="F22" s="16" t="n">
         <f aca="false">'Cash Flow'!F14</f>
-        <v>5606125</v>
+        <v>-39694875</v>
       </c>
       <c r="G22" s="16" t="n">
         <f aca="false">'Cash Flow'!G14</f>
-        <v>28163000</v>
+        <v>-35432500</v>
       </c>
       <c r="H22" s="16" t="n">
         <f aca="false">'Cash Flow'!H14</f>
-        <v>-40999650</v>
+        <v>-123142800</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B46" s="29" t="s">
-        <v>123</v>
+        <v>134</v>
       </c>
       <c r="C46" s="29"/>
       <c r="D46" s="29"/>

</xml_diff>